<commit_message>
recent models for sample, alongside posit connect stuff
</commit_message>
<xml_diff>
--- a/Open Data Dashboard/Databricks/ae outputs/hospital_model_performance_no.xlsx
+++ b/Open Data Dashboard/Databricks/ae outputs/hospital_model_performance_no.xlsx
@@ -408,10 +408,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>45.23485387719025</v>
+        <v>46.49433325440703</v>
       </c>
       <c r="C2">
-        <v>0.6989154562235046</v>
+        <v>0.6821588981117277</v>
       </c>
       <c r="D2">
         <v>1211.402777777778</v>
@@ -420,7 +420,7 @@
         <v>500</v>
       </c>
       <c r="F2">
-        <v>0.03734088670340512</v>
+        <v>0.03838057342059029</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>34.0691210919662</v>
+        <v>34.01547793850995</v>
       </c>
       <c r="C3">
-        <v>0.6541191562167383</v>
+        <v>0.6562063656861638</v>
       </c>
       <c r="D3">
         <v>644.4583333333334</v>
@@ -457,7 +457,7 @@
         <v>500</v>
       </c>
       <c r="F3">
-        <v>0.0528647382302443</v>
+        <v>0.05278150064810491</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -482,10 +482,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>29.46077651623655</v>
+        <v>30.34848576287424</v>
       </c>
       <c r="C4">
-        <v>0.5666189252393639</v>
+        <v>0.5435389768111231</v>
       </c>
       <c r="D4">
         <v>629.8243243243244</v>
@@ -494,7 +494,7 @@
         <v>500</v>
       </c>
       <c r="F4">
-        <v>0.0467761808784411</v>
+        <v>0.04818563620170133</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>15.75797306632392</v>
+        <v>16.26092344233312</v>
       </c>
       <c r="C5">
-        <v>0.5283775531413354</v>
+        <v>0.5119458329799657</v>
       </c>
       <c r="D5">
         <v>176.1081081081081</v>
@@ -531,7 +531,7 @@
         <v>500</v>
       </c>
       <c r="F5">
-        <v>0.08947897536126229</v>
+        <v>0.09233489370262819</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -556,10 +556,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>28.59450435026173</v>
+        <v>30.19176859166994</v>
       </c>
       <c r="C6">
-        <v>0.3721725778803721</v>
+        <v>0.320100996694096</v>
       </c>
       <c r="D6">
         <v>560.4324324324324</v>
@@ -568,7 +568,7 @@
         <v>500</v>
       </c>
       <c r="F6">
-        <v>0.05102221551696007</v>
+        <v>0.05387227227487404</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -593,10 +593,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>35.42711448703533</v>
+        <v>36.94602427452214</v>
       </c>
       <c r="C7">
-        <v>0.6557951618951233</v>
+        <v>0.6262827666645755</v>
       </c>
       <c r="D7">
         <v>1077.837837837838</v>
@@ -605,7 +605,7 @@
         <v>500</v>
       </c>
       <c r="F7">
-        <v>0.03286868696139186</v>
+        <v>0.03427790617245033</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>40.23741236752557</v>
+        <v>39.77712353590125</v>
       </c>
       <c r="C8">
-        <v>0.7440745830343477</v>
+        <v>0.7499037485586925</v>
       </c>
       <c r="D8">
         <v>1331.351351351351</v>
@@ -642,7 +642,7 @@
         <v>500</v>
       </c>
       <c r="F8">
-        <v>0.03022298533492583</v>
+        <v>0.02987725478742075</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="B9">
-        <v>62.47404553171553</v>
+        <v>65.78741069155895</v>
       </c>
       <c r="C9">
-        <v>0.5375810192240882</v>
+        <v>0.4959773477435798</v>
       </c>
       <c r="D9">
         <v>1606.959459459459</v>
@@ -679,7 +679,7 @@
         <v>500</v>
       </c>
       <c r="F9">
-        <v>0.03887717587644073</v>
+        <v>0.04093906059938075</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -704,10 +704,10 @@
         </is>
       </c>
       <c r="B10">
-        <v>60.75749841149079</v>
+        <v>64.99804999798062</v>
       </c>
       <c r="C10">
-        <v>0.570033399963161</v>
+        <v>0.5201814343748333</v>
       </c>
       <c r="D10">
         <v>1936.189189189189</v>
@@ -716,7 +716,7 @@
         <v>500</v>
       </c>
       <c r="F10">
-        <v>0.03137993887721994</v>
+        <v>0.03357009240672375</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -741,10 +741,10 @@
         </is>
       </c>
       <c r="B11">
-        <v>97.07353915696984</v>
+        <v>97.63220439597237</v>
       </c>
       <c r="C11">
-        <v>0.6862756389626397</v>
+        <v>0.6830135580954528</v>
       </c>
       <c r="D11">
         <v>1444.905405405405</v>
@@ -753,7 +753,7 @@
         <v>500</v>
       </c>
       <c r="F11">
-        <v>0.06718331787936897</v>
+        <v>0.06756996273301305</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="B12">
-        <v>15.12283634184477</v>
+        <v>15.68875753180156</v>
       </c>
       <c r="C12">
-        <v>0.4870643810208503</v>
+        <v>0.4655327756397026</v>
       </c>
       <c r="D12">
         <v>185.3108108108108</v>
@@ -790,7 +790,7 @@
         <v>500</v>
       </c>
       <c r="F12">
-        <v>0.08160795517366827</v>
+        <v>0.08466185789785717</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="B13">
-        <v>30.57972623760867</v>
+        <v>30.99356563201531</v>
       </c>
       <c r="C13">
-        <v>0.7398698511731722</v>
+        <v>0.7348719147065071</v>
       </c>
       <c r="D13">
         <v>763.9324324324324</v>
@@ -827,7 +827,7 @@
         <v>500</v>
       </c>
       <c r="F13">
-        <v>0.04002935984827867</v>
+        <v>0.04057108235780604</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -852,10 +852,10 @@
         </is>
       </c>
       <c r="B14">
-        <v>16.15089647403337</v>
+        <v>16.30791036801128</v>
       </c>
       <c r="C14">
-        <v>0.7818083609621532</v>
+        <v>0.7763808732130766</v>
       </c>
       <c r="D14">
         <v>179.5405405405405</v>
@@ -864,7 +864,7 @@
         <v>500</v>
       </c>
       <c r="F14">
-        <v>0.08995682214951596</v>
+        <v>0.09083135384862522</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -889,10 +889,10 @@
         </is>
       </c>
       <c r="B15">
-        <v>40.66705813095449</v>
+        <v>41.91726927992283</v>
       </c>
       <c r="C15">
-        <v>0.6732448264643847</v>
+        <v>0.6533371829860668</v>
       </c>
       <c r="D15">
         <v>1240.108108108108</v>
@@ -901,7 +901,7 @@
         <v>500</v>
       </c>
       <c r="F15">
-        <v>0.03279315558463334</v>
+        <v>0.03380130248795102</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -926,10 +926,10 @@
         </is>
       </c>
       <c r="B16">
-        <v>45.59904885649723</v>
+        <v>46.04622434982161</v>
       </c>
       <c r="C16">
-        <v>0.6543913921854482</v>
+        <v>0.648104905569906</v>
       </c>
       <c r="D16">
         <v>1222.675675675676</v>
@@ -938,7 +938,7 @@
         <v>500</v>
       </c>
       <c r="F16">
-        <v>0.0372944761752116</v>
+        <v>0.03766021134294303</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -963,10 +963,10 @@
         </is>
       </c>
       <c r="B17">
-        <v>45.77770468109137</v>
+        <v>45.50079377860992</v>
       </c>
       <c r="C17">
-        <v>0.6295116000437658</v>
+        <v>0.6342262646132728</v>
       </c>
       <c r="D17">
         <v>1347</v>
@@ -975,7 +975,7 @@
         <v>500</v>
       </c>
       <c r="F17">
-        <v>0.0339849329481005</v>
+        <v>0.03377935692547136</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1000,10 +1000,10 @@
         </is>
       </c>
       <c r="B18">
-        <v>34.49686446361387</v>
+        <v>35.4351804396951</v>
       </c>
       <c r="C18">
-        <v>0.7587597735584393</v>
+        <v>0.7455295299677986</v>
       </c>
       <c r="D18">
         <v>1091.013513513514</v>
@@ -1012,7 +1012,7 @@
         <v>500</v>
       </c>
       <c r="F18">
-        <v>0.03161909915535303</v>
+        <v>0.03247913980971619</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="B19">
-        <v>34.21444283503374</v>
+        <v>33.71704586418945</v>
       </c>
       <c r="C19">
-        <v>0.6341822883690409</v>
+        <v>0.6471452666401072</v>
       </c>
       <c r="D19">
         <v>351.1486486486486</v>
@@ -1049,7 +1049,7 @@
         <v>500</v>
       </c>
       <c r="F19">
-        <v>0.09743578101953036</v>
+        <v>0.09601929551472078</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1074,10 +1074,10 @@
         </is>
       </c>
       <c r="B20">
-        <v>29.42182156216352</v>
+        <v>29.6418154030207</v>
       </c>
       <c r="C20">
-        <v>0.652122715290918</v>
+        <v>0.6491038354465648</v>
       </c>
       <c r="D20">
         <v>506.5405405405405</v>
@@ -1086,7 +1086,7 @@
         <v>500</v>
       </c>
       <c r="F20">
-        <v>0.05808384365596255</v>
+        <v>0.05851815013935365</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1111,10 +1111,10 @@
         </is>
       </c>
       <c r="B21">
-        <v>14.3414439735985</v>
+        <v>15.05990891862479</v>
       </c>
       <c r="C21">
-        <v>0.5147291432227826</v>
+        <v>0.4852173598998777</v>
       </c>
       <c r="D21">
         <v>147.2027027027027</v>
@@ -1123,7 +1123,7 @@
         <v>500</v>
       </c>
       <c r="F21">
-        <v>0.09742649904032767</v>
+        <v>0.1023072854106522</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="B22">
-        <v>35.92200439071657</v>
+        <v>36.95858047908116</v>
       </c>
       <c r="C22">
-        <v>0.73906517650557</v>
+        <v>0.7243823446853056</v>
       </c>
       <c r="D22">
         <v>1100.662162162162</v>
@@ -1160,7 +1160,7 @@
         <v>500</v>
       </c>
       <c r="F22">
-        <v>0.03263672144425379</v>
+        <v>0.03357849642662288</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1185,10 +1185,10 @@
         </is>
       </c>
       <c r="B23">
-        <v>74.40064281649174</v>
+        <v>75.94759892022134</v>
       </c>
       <c r="C23">
-        <v>0.6593232807841106</v>
+        <v>0.6398567244992773</v>
       </c>
       <c r="D23">
         <v>2402.175675675676</v>
@@ -1197,7 +1197,7 @@
         <v>500</v>
       </c>
       <c r="F23">
-        <v>0.03097219057285</v>
+        <v>0.03161617182675828</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1222,10 +1222,10 @@
         </is>
       </c>
       <c r="B24">
-        <v>76.97835909669762</v>
+        <v>77.25347467497163</v>
       </c>
       <c r="C24">
-        <v>0.6819447115296725</v>
+        <v>0.6815135103524624</v>
       </c>
       <c r="D24">
         <v>1028.351351351351</v>
@@ -1234,7 +1234,7 @@
         <v>500</v>
       </c>
       <c r="F24">
-        <v>0.07485608784929465</v>
+        <v>0.07512361857010567</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="B25">
-        <v>41.56950225708304</v>
+        <v>42.03585644409962</v>
       </c>
       <c r="C25">
-        <v>0.6836053762296851</v>
+        <v>0.6767425214247695</v>
       </c>
       <c r="D25">
         <v>1186.959459459459</v>
@@ -1271,7 +1271,7 @@
         <v>500</v>
       </c>
       <c r="F25">
-        <v>0.0350218382993584</v>
+        <v>0.03541473645885321</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1296,10 +1296,10 @@
         </is>
       </c>
       <c r="B26">
-        <v>26.36145520417057</v>
+        <v>27.31490451493142</v>
       </c>
       <c r="C26">
-        <v>0.6048954121527488</v>
+        <v>0.577309610159242</v>
       </c>
       <c r="D26">
         <v>450.027027027027</v>
@@ -1308,7 +1308,7 @@
         <v>500</v>
       </c>
       <c r="F26">
-        <v>0.0585774933970519</v>
+        <v>0.06069614239700094</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1333,10 +1333,10 @@
         </is>
       </c>
       <c r="B27">
-        <v>37.67373288450491</v>
+        <v>37.95973600363648</v>
       </c>
       <c r="C27">
-        <v>0.6960688578196195</v>
+        <v>0.6902709772423981</v>
       </c>
       <c r="D27">
         <v>1172.797297297297</v>
@@ -1345,7 +1345,7 @@
         <v>500</v>
       </c>
       <c r="F27">
-        <v>0.03212297041553877</v>
+        <v>0.0323668344829191</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1370,10 +1370,10 @@
         </is>
       </c>
       <c r="B28">
-        <v>11.37632767444268</v>
+        <v>11.61618883957597</v>
       </c>
       <c r="C28">
-        <v>0.5018868813436187</v>
+        <v>0.5045168944900501</v>
       </c>
       <c r="D28">
         <v>111.3108108108108</v>
@@ -1382,7 +1382,7 @@
         <v>500</v>
       </c>
       <c r="F28">
-        <v>0.1022032594280392</v>
+        <v>0.1043581369586769</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1407,10 +1407,10 @@
         </is>
       </c>
       <c r="B29">
-        <v>18.47643094162426</v>
+        <v>18.98196180970888</v>
       </c>
       <c r="C29">
-        <v>0.4437473583673844</v>
+        <v>0.4225009942085635</v>
       </c>
       <c r="D29">
         <v>264.6216216216216</v>
@@ -1419,7 +1419,7 @@
         <v>500</v>
       </c>
       <c r="F29">
-        <v>0.0698220758696862</v>
+        <v>0.07173246726169222</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1444,10 +1444,10 @@
         </is>
       </c>
       <c r="B30">
-        <v>33.5404909909284</v>
+        <v>32.46914639837345</v>
       </c>
       <c r="C30">
-        <v>0.7689789710837758</v>
+        <v>0.7831244168701935</v>
       </c>
       <c r="D30">
         <v>698.0405405405405</v>
@@ -1456,7 +1456,7 @@
         <v>500</v>
       </c>
       <c r="F30">
-        <v>0.04804948859410902</v>
+        <v>0.0465147000964018</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1481,10 +1481,10 @@
         </is>
       </c>
       <c r="B31">
-        <v>13.96234452562645</v>
+        <v>14.26283739718588</v>
       </c>
       <c r="C31">
-        <v>0.4554497801196244</v>
+        <v>0.4494042352585648</v>
       </c>
       <c r="D31">
         <v>161.3108108108108</v>
@@ -1493,7 +1493,7 @@
         <v>500</v>
       </c>
       <c r="F31">
-        <v>0.08655554116581698</v>
+        <v>0.08841836034110373</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1518,10 +1518,10 @@
         </is>
       </c>
       <c r="B32">
-        <v>38.77187246698245</v>
+        <v>37.43070039517617</v>
       </c>
       <c r="C32">
-        <v>0.7822627608575428</v>
+        <v>0.7981094187109143</v>
       </c>
       <c r="D32">
         <v>1211.402777777778</v>
@@ -1530,7 +1530,7 @@
         <v>1000</v>
       </c>
       <c r="F32">
-        <v>0.03200576486881297</v>
+        <v>0.03089864170844962</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1555,10 +1555,10 @@
         </is>
       </c>
       <c r="B33">
-        <v>33.92157600410846</v>
+        <v>34.12972028631665</v>
       </c>
       <c r="C33">
-        <v>0.657245728355035</v>
+        <v>0.6513166645527161</v>
       </c>
       <c r="D33">
         <v>644.4583333333334</v>
@@ -1567,7 +1567,7 @@
         <v>1000</v>
       </c>
       <c r="F33">
-        <v>0.05263579389012756</v>
+        <v>0.05295876943632247</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1592,10 +1592,10 @@
         </is>
       </c>
       <c r="B34">
-        <v>29.63460840962281</v>
+        <v>29.235319694997</v>
       </c>
       <c r="C34">
-        <v>0.5619254155114285</v>
+        <v>0.5700473861276555</v>
       </c>
       <c r="D34">
         <v>629.8243243243244</v>
@@ -1604,7 +1604,7 @@
         <v>1000</v>
       </c>
       <c r="F34">
-        <v>0.0470521814815819</v>
+        <v>0.04641821308880163</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1629,10 +1629,10 @@
         </is>
       </c>
       <c r="B35">
-        <v>16.48303702362585</v>
+        <v>15.42433743161232</v>
       </c>
       <c r="C35">
-        <v>0.4879825206309807</v>
+        <v>0.5403287344913315</v>
       </c>
       <c r="D35">
         <v>176.1081081081081</v>
@@ -1641,7 +1641,7 @@
         <v>1000</v>
       </c>
       <c r="F35">
-        <v>0.09359612797332051</v>
+        <v>0.087584482039542</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1666,10 +1666,10 @@
         </is>
       </c>
       <c r="B36">
-        <v>29.5892626933958</v>
+        <v>29.60163663819558</v>
       </c>
       <c r="C36">
-        <v>0.3372139181841807</v>
+        <v>0.3394534400179265</v>
       </c>
       <c r="D36">
         <v>560.4324324324324</v>
@@ -1678,7 +1678,7 @@
         <v>1000</v>
       </c>
       <c r="F36">
-        <v>0.05279719905746743</v>
+        <v>0.0528192783378297</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1703,10 +1703,10 @@
         </is>
       </c>
       <c r="B37">
-        <v>31.57557924690478</v>
+        <v>31.81916908306097</v>
       </c>
       <c r="C37">
-        <v>0.7265421663804543</v>
+        <v>0.7230866892034168</v>
       </c>
       <c r="D37">
         <v>1077.837837837838</v>
@@ -1715,7 +1715,7 @@
         <v>1000</v>
       </c>
       <c r="F37">
-        <v>0.02929529669346732</v>
+        <v>0.02952129528769448</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="B38">
-        <v>33.95046584346628</v>
+        <v>33.61603636177525</v>
       </c>
       <c r="C38">
-        <v>0.8181372680150462</v>
+        <v>0.8232276470009428</v>
       </c>
       <c r="D38">
         <v>1331.351351351351</v>
@@ -1752,7 +1752,7 @@
         <v>1000</v>
       </c>
       <c r="F38">
-        <v>0.02550075591165758</v>
+        <v>0.02524956040165823</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1777,10 +1777,10 @@
         </is>
       </c>
       <c r="B39">
-        <v>61.41677390437512</v>
+        <v>59.64446820945306</v>
       </c>
       <c r="C39">
-        <v>0.5553851362043249</v>
+        <v>0.576210432833965</v>
       </c>
       <c r="D39">
         <v>1606.959459459459</v>
@@ -1789,7 +1789,7 @@
         <v>1000</v>
       </c>
       <c r="F39">
-        <v>0.03821924289554521</v>
+        <v>0.03711634905183978</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1814,10 +1814,10 @@
         </is>
       </c>
       <c r="B40">
-        <v>61.25954803109533</v>
+        <v>58.393204060884</v>
       </c>
       <c r="C40">
-        <v>0.5717476262982465</v>
+        <v>0.6030583708808438</v>
       </c>
       <c r="D40">
         <v>1936.189189189189</v>
@@ -1826,7 +1826,7 @@
         <v>1000</v>
       </c>
       <c r="F40">
-        <v>0.03163923668882211</v>
+        <v>0.03015883178509901</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1851,10 +1851,10 @@
         </is>
       </c>
       <c r="B41">
-        <v>82.72331548869717</v>
+        <v>81.39944543352939</v>
       </c>
       <c r="C41">
-        <v>0.7723099155609841</v>
+        <v>0.780635543536271</v>
       </c>
       <c r="D41">
         <v>1444.905405405405</v>
@@ -1863,7 +1863,7 @@
         <v>1000</v>
       </c>
       <c r="F41">
-        <v>0.05725171708765738</v>
+        <v>0.05633548405938082</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1888,10 +1888,10 @@
         </is>
       </c>
       <c r="B42">
-        <v>15.57604989168016</v>
+        <v>15.10085337697159</v>
       </c>
       <c r="C42">
-        <v>0.4580316369602181</v>
+        <v>0.4822744933172856</v>
       </c>
       <c r="D42">
         <v>185.3108108108108</v>
@@ -1900,7 +1900,7 @@
         <v>1000</v>
       </c>
       <c r="F42">
-        <v>0.0840536492368068</v>
+        <v>0.08148932763770857</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="B43">
-        <v>31.16306600333486</v>
+        <v>30.77270973038397</v>
       </c>
       <c r="C43">
-        <v>0.7379069367012493</v>
+        <v>0.7371224447373209</v>
       </c>
       <c r="D43">
         <v>763.9324324324324</v>
@@ -1937,7 +1937,7 @@
         <v>1000</v>
       </c>
       <c r="F43">
-        <v>0.04079296110535422</v>
+        <v>0.04028197838439819</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1962,10 +1962,10 @@
         </is>
       </c>
       <c r="B44">
-        <v>16.37535211898211</v>
+        <v>16.18067092337338</v>
       </c>
       <c r="C44">
-        <v>0.7724805637830803</v>
+        <v>0.7752397310701824</v>
       </c>
       <c r="D44">
         <v>179.5405405405405</v>
@@ -1974,7 +1974,7 @@
         <v>1000</v>
       </c>
       <c r="F44">
-        <v>0.09120698907155475</v>
+        <v>0.09012265906440088</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -1999,10 +1999,10 @@
         </is>
       </c>
       <c r="B45">
-        <v>35.04120525253303</v>
+        <v>34.32261359275291</v>
       </c>
       <c r="C45">
-        <v>0.7542309024606907</v>
+        <v>0.7646077043633425</v>
       </c>
       <c r="D45">
         <v>1240.108108108108</v>
@@ -2011,7 +2011,7 @@
         <v>1000</v>
       </c>
       <c r="F45">
-        <v>0.02825657297410257</v>
+        <v>0.02767711409057313</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         </is>
       </c>
       <c r="B46">
-        <v>39.42159737425224</v>
+        <v>37.36359466476471</v>
       </c>
       <c r="C46">
-        <v>0.7391433110485278</v>
+        <v>0.7661582252179419</v>
       </c>
       <c r="D46">
         <v>1222.675675675676</v>
@@ -2048,7 +2048,7 @@
         <v>1000</v>
       </c>
       <c r="F46">
-        <v>0.03224207216886608</v>
+        <v>0.03055887624828786</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2073,10 +2073,10 @@
         </is>
       </c>
       <c r="B47">
-        <v>38.69200782966568</v>
+        <v>37.61433147869957</v>
       </c>
       <c r="C47">
-        <v>0.7365261563977332</v>
+        <v>0.7528224930055586</v>
       </c>
       <c r="D47">
         <v>1347</v>
@@ -2085,7 +2085,7 @@
         <v>1000</v>
       </c>
       <c r="F47">
-        <v>0.02872457893813339</v>
+        <v>0.02792452225590169</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2110,10 +2110,10 @@
         </is>
       </c>
       <c r="B48">
-        <v>29.57924298221318</v>
+        <v>30.07142673086196</v>
       </c>
       <c r="C48">
-        <v>0.8248265228378078</v>
+        <v>0.820668944974017</v>
       </c>
       <c r="D48">
         <v>1091.013513513514</v>
@@ -2122,7 +2122,7 @@
         <v>1000</v>
       </c>
       <c r="F48">
-        <v>0.02711171091452004</v>
+        <v>0.02756283616874695</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2147,10 +2147,10 @@
         </is>
       </c>
       <c r="B49">
-        <v>34.12363678934803</v>
+        <v>33.27196367040963</v>
       </c>
       <c r="C49">
-        <v>0.6394412700226877</v>
+        <v>0.6503539029728914</v>
       </c>
       <c r="D49">
         <v>351.1486486486486</v>
@@ -2159,7 +2159,7 @@
         <v>1000</v>
       </c>
       <c r="F49">
-        <v>0.09717718385267479</v>
+        <v>0.09475179186493411</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2184,10 +2184,10 @@
         </is>
       </c>
       <c r="B50">
-        <v>29.43357807420023</v>
+        <v>29.40605557924493</v>
       </c>
       <c r="C50">
-        <v>0.6511598599998994</v>
+        <v>0.6497208035636731</v>
       </c>
       <c r="D50">
         <v>506.5405405405405</v>
@@ -2196,7 +2196,7 @@
         <v>1000</v>
       </c>
       <c r="F50">
-        <v>0.05810705307573411</v>
+        <v>0.05805271883641355</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="B51">
-        <v>14.61084463699289</v>
+        <v>14.80995975038469</v>
       </c>
       <c r="C51">
-        <v>0.4904822115677073</v>
+        <v>0.4789090452765793</v>
       </c>
       <c r="D51">
         <v>147.2027027027027</v>
@@ -2233,7 +2233,7 @@
         <v>1000</v>
       </c>
       <c r="F51">
-        <v>0.09925663298792564</v>
+        <v>0.1006092923463203</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2258,10 +2258,10 @@
         </is>
       </c>
       <c r="B52">
-        <v>31.28499021752662</v>
+        <v>31.7055712171958</v>
       </c>
       <c r="C52">
-        <v>0.8021242127651277</v>
+        <v>0.7965643473375706</v>
       </c>
       <c r="D52">
         <v>1100.662162162162</v>
@@ -2270,7 +2270,7 @@
         <v>1000</v>
       </c>
       <c r="F52">
-        <v>0.02842379005386156</v>
+        <v>0.02880590639630308</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2295,10 +2295,10 @@
         </is>
       </c>
       <c r="B53">
-        <v>74.95200543248018</v>
+        <v>74.74932298385046</v>
       </c>
       <c r="C53">
-        <v>0.6417052681935641</v>
+        <v>0.6450105678305423</v>
       </c>
       <c r="D53">
         <v>2402.175675675676</v>
@@ -2307,7 +2307,7 @@
         <v>1000</v>
       </c>
       <c r="F53">
-        <v>0.03120171692330451</v>
+        <v>0.03111734239121592</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2332,10 +2332,10 @@
         </is>
       </c>
       <c r="B54">
-        <v>65.85386010979251</v>
+        <v>63.96362866414099</v>
       </c>
       <c r="C54">
-        <v>0.7656183482913402</v>
+        <v>0.7802554443685467</v>
       </c>
       <c r="D54">
         <v>1028.351351351351</v>
@@ -2344,7 +2344,7 @@
         <v>1000</v>
       </c>
       <c r="F54">
-        <v>0.06403828810382199</v>
+        <v>0.062200169796137</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2369,10 +2369,10 @@
         </is>
       </c>
       <c r="B55">
-        <v>35.07227047848739</v>
+        <v>33.57250390644953</v>
       </c>
       <c r="C55">
-        <v>0.7729934775329712</v>
+        <v>0.7930504854508468</v>
       </c>
       <c r="D55">
         <v>1186.959459459459</v>
@@ -2381,7 +2381,7 @@
         <v>1000</v>
       </c>
       <c r="F55">
-        <v>0.02954799357213032</v>
+        <v>0.02828445709657045</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2406,10 +2406,10 @@
         </is>
       </c>
       <c r="B56">
-        <v>27.10328260370671</v>
+        <v>26.98490438514023</v>
       </c>
       <c r="C56">
-        <v>0.5842376264063691</v>
+        <v>0.5932852921038002</v>
       </c>
       <c r="D56">
         <v>450.027027027027</v>
@@ -2418,7 +2418,7 @@
         <v>1000</v>
       </c>
       <c r="F56">
-        <v>0.06022589972597132</v>
+        <v>0.05996285281665897</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2443,10 +2443,10 @@
         </is>
       </c>
       <c r="B57">
-        <v>32.30604467957674</v>
+        <v>30.71888335182818</v>
       </c>
       <c r="C57">
-        <v>0.7742513274575649</v>
+        <v>0.796400778676345</v>
       </c>
       <c r="D57">
         <v>1172.797297297297</v>
@@ -2455,7 +2455,7 @@
         <v>1000</v>
       </c>
       <c r="F57">
-        <v>0.02754614523245047</v>
+        <v>0.02619283265967582</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2480,10 +2480,10 @@
         </is>
       </c>
       <c r="B58">
-        <v>11.3377278621331</v>
+        <v>11.48916437067259</v>
       </c>
       <c r="C58">
-        <v>0.4787127513664166</v>
+        <v>0.4579044213860243</v>
       </c>
       <c r="D58">
         <v>111.3108108108108</v>
@@ -2492,7 +2492,7 @@
         <v>1000</v>
       </c>
       <c r="F58">
-        <v>0.1018564843751183</v>
+        <v>0.1032169677588651</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2517,10 +2517,10 @@
         </is>
       </c>
       <c r="B59">
-        <v>18.54728067649277</v>
+        <v>18.25119104466176</v>
       </c>
       <c r="C59">
-        <v>0.4376979055002164</v>
+        <v>0.4518890759442061</v>
       </c>
       <c r="D59">
         <v>264.6216216216216</v>
@@ -2529,7 +2529,7 @@
         <v>1000</v>
       </c>
       <c r="F59">
-        <v>0.07008981565011056</v>
+        <v>0.0689708986469702</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2554,10 +2554,10 @@
         </is>
       </c>
       <c r="B60">
-        <v>32.66427326359256</v>
+        <v>32.54464973220322</v>
       </c>
       <c r="C60">
-        <v>0.78110069214599</v>
+        <v>0.7816992618022339</v>
       </c>
       <c r="D60">
         <v>698.0405405405405</v>
@@ -2566,7 +2566,7 @@
         <v>1000</v>
       </c>
       <c r="F60">
-        <v>0.04679423524355531</v>
+        <v>0.04662286477946062</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2591,10 +2591,10 @@
         </is>
       </c>
       <c r="B61">
-        <v>14.51029382495368</v>
+        <v>14.35533520828302</v>
       </c>
       <c r="C61">
-        <v>0.4172714017071864</v>
+        <v>0.4201487205631637</v>
       </c>
       <c r="D61">
         <v>161.3108108108108</v>
@@ -2603,7 +2603,7 @@
         <v>1000</v>
       </c>
       <c r="F61">
-        <v>0.08995239532936014</v>
+        <v>0.08899177393088244</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2628,10 +2628,10 @@
         </is>
       </c>
       <c r="B62">
-        <v>30.25951554643397</v>
+        <v>30.98257107242751</v>
       </c>
       <c r="C62">
-        <v>0.8766006104451975</v>
+        <v>0.8694321853423094</v>
       </c>
       <c r="D62">
         <v>1211.402777777778</v>
@@ -2640,7 +2640,7 @@
         <v>2000</v>
       </c>
       <c r="F62">
-        <v>0.02497890553127396</v>
+        <v>0.02557578011275703</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2665,10 +2665,10 @@
         </is>
       </c>
       <c r="B63">
-        <v>32.80144827445333</v>
+        <v>32.54172330642157</v>
       </c>
       <c r="C63">
-        <v>0.6761318233857564</v>
+        <v>0.6796035355536136</v>
       </c>
       <c r="D63">
         <v>644.4583333333334</v>
@@ -2677,7 +2677,7 @@
         <v>2000</v>
       </c>
       <c r="F63">
-        <v>0.05089770211333031</v>
+        <v>0.05049468929683311</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2702,10 +2702,10 @@
         </is>
       </c>
       <c r="B64">
-        <v>27.59972760119804</v>
+        <v>27.82743915774003</v>
       </c>
       <c r="C64">
-        <v>0.6138505782937393</v>
+        <v>0.6071368363551288</v>
       </c>
       <c r="D64">
         <v>629.8243243243244</v>
@@ -2714,7 +2714,7 @@
         <v>2000</v>
       </c>
       <c r="F64">
-        <v>0.04382131101526926</v>
+        <v>0.04418285874810141</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2739,10 +2739,10 @@
         </is>
       </c>
       <c r="B65">
-        <v>15.85613156000613</v>
+        <v>15.41097957806962</v>
       </c>
       <c r="C65">
-        <v>0.5162866400312016</v>
+        <v>0.5420748702015589</v>
       </c>
       <c r="D65">
         <v>176.1081081081081</v>
@@ -2751,7 +2751,7 @@
         <v>2000</v>
       </c>
       <c r="F65">
-        <v>0.09003635170660323</v>
+        <v>0.08750863173550889</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2776,10 +2776,10 @@
         </is>
       </c>
       <c r="B66">
-        <v>28.90301723419028</v>
+        <v>28.13555201545193</v>
       </c>
       <c r="C66">
-        <v>0.3506593265519375</v>
+        <v>0.3843849010691283</v>
       </c>
       <c r="D66">
         <v>560.4324324324324</v>
@@ -2788,7 +2788,7 @@
         <v>2000</v>
       </c>
       <c r="F66">
-        <v>0.05157270629171685</v>
+        <v>0.05020329015102823</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2813,10 +2813,10 @@
         </is>
       </c>
       <c r="B67">
-        <v>26.59613508581764</v>
+        <v>26.49464822835969</v>
       </c>
       <c r="C67">
-        <v>0.811072266682514</v>
+        <v>0.812609325486674</v>
       </c>
       <c r="D67">
         <v>1077.837837837838</v>
@@ -2825,7 +2825,7 @@
         <v>2000</v>
       </c>
       <c r="F67">
-        <v>0.02467545130830624</v>
+        <v>0.02458129349170783</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2850,10 +2850,10 @@
         </is>
       </c>
       <c r="B68">
-        <v>26.48985909340352</v>
+        <v>27.51036315680549</v>
       </c>
       <c r="C68">
-        <v>0.8945281472699069</v>
+        <v>0.883112081580299</v>
       </c>
       <c r="D68">
         <v>1331.351351351351</v>
@@ -2862,7 +2862,7 @@
         <v>2000</v>
       </c>
       <c r="F68">
-        <v>0.01989697089841515</v>
+        <v>0.02066348836382061</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2887,10 +2887,10 @@
         </is>
       </c>
       <c r="B69">
-        <v>52.33776552183924</v>
+        <v>52.74179640798228</v>
       </c>
       <c r="C69">
-        <v>0.6653697521736837</v>
+        <v>0.6613793879243559</v>
       </c>
       <c r="D69">
         <v>1606.959459459459</v>
@@ -2899,7 +2899,7 @@
         <v>2000</v>
       </c>
       <c r="F69">
-        <v>0.03256943740164071</v>
+        <v>0.03282086308868258</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         </is>
       </c>
       <c r="B70">
-        <v>53.71286588946593</v>
+        <v>53.82206564591981</v>
       </c>
       <c r="C70">
-        <v>0.6633195557419974</v>
+        <v>0.6630486716166363</v>
       </c>
       <c r="D70">
         <v>1936.189189189189</v>
@@ -2936,7 +2936,7 @@
         <v>2000</v>
       </c>
       <c r="F70">
-        <v>0.02774153795991345</v>
+        <v>0.02779793728135559</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2961,10 +2961,10 @@
         </is>
       </c>
       <c r="B71">
-        <v>66.34972440857985</v>
+        <v>65.44711201333412</v>
       </c>
       <c r="C71">
-        <v>0.8545072861055724</v>
+        <v>0.8595172052506872</v>
       </c>
       <c r="D71">
         <v>1444.905405405405</v>
@@ -2973,7 +2973,7 @@
         <v>2000</v>
       </c>
       <c r="F71">
-        <v>0.04591977036030516</v>
+        <v>0.04529508421000837</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2998,10 +2998,10 @@
         </is>
       </c>
       <c r="B72">
-        <v>15.03514905308365</v>
+        <v>15.15617293645336</v>
       </c>
       <c r="C72">
-        <v>0.4833301995914936</v>
+        <v>0.4757818434437468</v>
       </c>
       <c r="D72">
         <v>185.3108108108108</v>
@@ -3010,7 +3010,7 @@
         <v>2000</v>
       </c>
       <c r="F72">
-        <v>0.08113476481646542</v>
+        <v>0.08178785074728713</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -3035,10 +3035,10 @@
         </is>
       </c>
       <c r="B73">
-        <v>29.75907783646485</v>
+        <v>28.68408960148722</v>
       </c>
       <c r="C73">
-        <v>0.754568083067539</v>
+        <v>0.7712516791634009</v>
       </c>
       <c r="D73">
         <v>763.9324324324324</v>
@@ -3047,7 +3047,7 @@
         <v>2000</v>
       </c>
       <c r="F73">
-        <v>0.03895511772122198</v>
+        <v>0.03754794060798596</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -3072,10 +3072,10 @@
         </is>
       </c>
       <c r="B74">
-        <v>16.41498104277835</v>
+        <v>15.69313616223397</v>
       </c>
       <c r="C74">
-        <v>0.7688052330914179</v>
+        <v>0.7896730680315381</v>
       </c>
       <c r="D74">
         <v>179.5405405405405</v>
@@ -3084,7 +3084,7 @@
         <v>2000</v>
       </c>
       <c r="F74">
-        <v>0.09142771316917038</v>
+        <v>0.08740720126488889</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -3109,10 +3109,10 @@
         </is>
       </c>
       <c r="B75">
-        <v>27.56523143555312</v>
+        <v>27.75822692020073</v>
       </c>
       <c r="C75">
-        <v>0.8510913772889273</v>
+        <v>0.8478280398064393</v>
       </c>
       <c r="D75">
         <v>1240.108108108108</v>
@@ -3121,7 +3121,7 @@
         <v>2000</v>
       </c>
       <c r="F75">
-        <v>0.02222808741860922</v>
+        <v>0.0223837153702255</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -3146,10 +3146,10 @@
         </is>
       </c>
       <c r="B76">
-        <v>29.85878253604825</v>
+        <v>32.17273994992841</v>
       </c>
       <c r="C76">
-        <v>0.8534878147275439</v>
+        <v>0.8280217907046893</v>
       </c>
       <c r="D76">
         <v>1222.675675675676</v>
@@ -3158,7 +3158,7 @@
         <v>2000</v>
       </c>
       <c r="F76">
-        <v>0.02442085266769348</v>
+        <v>0.02631338840706804</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -3183,10 +3183,10 @@
         </is>
       </c>
       <c r="B77">
-        <v>30.69066106724678</v>
+        <v>31.23895231751002</v>
       </c>
       <c r="C77">
-        <v>0.8404152819927304</v>
+        <v>0.8359510721752518</v>
       </c>
       <c r="D77">
         <v>1347</v>
@@ -3195,7 +3195,7 @@
         <v>2000</v>
       </c>
       <c r="F77">
-        <v>0.02278445513529828</v>
+        <v>0.02319150134930217</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -3220,10 +3220,10 @@
         </is>
       </c>
       <c r="B78">
-        <v>26.53929005694762</v>
+        <v>26.32051891142917</v>
       </c>
       <c r="C78">
-        <v>0.8636841734798759</v>
+        <v>0.8659860576276368</v>
       </c>
       <c r="D78">
         <v>1091.013513513514</v>
@@ -3232,7 +3232,7 @@
         <v>2000</v>
       </c>
       <c r="F78">
-        <v>0.02432535411177462</v>
+        <v>0.02412483308906619</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3257,10 +3257,10 @@
         </is>
       </c>
       <c r="B79">
-        <v>34.10021184092822</v>
+        <v>33.9344599115403</v>
       </c>
       <c r="C79">
-        <v>0.6371955462402648</v>
+        <v>0.6403329357882862</v>
       </c>
       <c r="D79">
         <v>351.1486486486486</v>
@@ -3269,7 +3269,7 @@
         <v>2000</v>
       </c>
       <c r="F79">
-        <v>0.09711047435938767</v>
+        <v>0.09663844654431335</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3294,10 +3294,10 @@
         </is>
       </c>
       <c r="B80">
-        <v>29.26923224779322</v>
+        <v>29.03845077929634</v>
       </c>
       <c r="C80">
-        <v>0.6537594954543402</v>
+        <v>0.6587942991091279</v>
       </c>
       <c r="D80">
         <v>506.5405405405405</v>
@@ -3306,7 +3306,7 @@
         <v>2000</v>
       </c>
       <c r="F80">
-        <v>0.0577826055473455</v>
+        <v>0.05732700239216544</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3331,10 +3331,10 @@
         </is>
       </c>
       <c r="B81">
-        <v>14.64316319625801</v>
+        <v>14.21756839533312</v>
       </c>
       <c r="C81">
-        <v>0.4798191424032019</v>
+        <v>0.5114202278152459</v>
       </c>
       <c r="D81">
         <v>147.2027027027027</v>
@@ -3343,7 +3343,7 @@
         <v>2000</v>
       </c>
       <c r="F81">
-        <v>0.09947618438658704</v>
+        <v>0.09658496844346379</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -3368,10 +3368,10 @@
         </is>
       </c>
       <c r="B82">
-        <v>26.29429009721144</v>
+        <v>26.97254799227818</v>
       </c>
       <c r="C82">
-        <v>0.861938513662124</v>
+        <v>0.8540515915727648</v>
       </c>
       <c r="D82">
         <v>1100.662162162162</v>
@@ -3380,7 +3380,7 @@
         <v>2000</v>
       </c>
       <c r="F82">
-        <v>0.02388951941943605</v>
+        <v>0.02450574655831975</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -3405,10 +3405,10 @@
         </is>
       </c>
       <c r="B83">
-        <v>77.70590710347274</v>
+        <v>79.54137315715558</v>
       </c>
       <c r="C83">
-        <v>0.628232184325046</v>
+        <v>0.6171742943923701</v>
       </c>
       <c r="D83">
         <v>2402.175675675676</v>
@@ -3417,7 +3417,7 @@
         <v>2000</v>
       </c>
       <c r="F83">
-        <v>0.03234813668722038</v>
+        <v>0.03311222154257409</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -3442,10 +3442,10 @@
         </is>
       </c>
       <c r="B84">
-        <v>53.33413566519593</v>
+        <v>52.80584853628979</v>
       </c>
       <c r="C84">
-        <v>0.846139824580859</v>
+        <v>0.8488234063735719</v>
       </c>
       <c r="D84">
         <v>1028.351351351351</v>
@@ -3454,7 +3454,7 @@
         <v>2000</v>
       </c>
       <c r="F84">
-        <v>0.05186372886573234</v>
+        <v>0.05135000646121377</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3479,10 +3479,10 @@
         </is>
       </c>
       <c r="B85">
-        <v>27.27801648833279</v>
+        <v>27.47682887489076</v>
       </c>
       <c r="C85">
-        <v>0.8688272038516072</v>
+        <v>0.8661065784516144</v>
       </c>
       <c r="D85">
         <v>1186.959459459459</v>
@@ -3491,7 +3491,7 @@
         <v>2000</v>
       </c>
       <c r="F85">
-        <v>0.02298142221365773</v>
+        <v>0.02314891941415058</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -3516,10 +3516,10 @@
         </is>
       </c>
       <c r="B86">
-        <v>26.76628939282152</v>
+        <v>26.79611178772305</v>
       </c>
       <c r="C86">
-        <v>0.5867510286744704</v>
+        <v>0.5877627242370268</v>
       </c>
       <c r="D86">
         <v>450.027027027027</v>
@@ -3528,7 +3528,7 @@
         <v>2000</v>
       </c>
       <c r="F86">
-        <v>0.05947707089870855</v>
+        <v>0.05954333890731804</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3553,10 +3553,10 @@
         </is>
       </c>
       <c r="B87">
-        <v>24.82961421268421</v>
+        <v>24.50698692530622</v>
       </c>
       <c r="C87">
-        <v>0.8685860074509721</v>
+        <v>0.8714195759499956</v>
       </c>
       <c r="D87">
         <v>1172.797297297297</v>
@@ -3565,7 +3565,7 @@
         <v>2000</v>
       </c>
       <c r="F87">
-        <v>0.02117127509579352</v>
+        <v>0.02089618298215931</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3590,10 +3590,10 @@
         </is>
       </c>
       <c r="B88">
-        <v>11.10954006974615</v>
+        <v>11.12481367108188</v>
       </c>
       <c r="C88">
-        <v>0.4756118785506706</v>
+        <v>0.4775698796586616</v>
       </c>
       <c r="D88">
         <v>111.3108108108108</v>
@@ -3602,7 +3602,7 @@
         <v>2000</v>
       </c>
       <c r="F88">
-        <v>0.0998064787132712</v>
+        <v>0.09994369450771631</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -3627,10 +3627,10 @@
         </is>
       </c>
       <c r="B89">
-        <v>18.54077154337231</v>
+        <v>19.00401814455854</v>
       </c>
       <c r="C89">
-        <v>0.4393893030007361</v>
+        <v>0.4142442373724089</v>
       </c>
       <c r="D89">
         <v>264.6216216216216</v>
@@ -3639,7 +3639,7 @@
         <v>2000</v>
       </c>
       <c r="F89">
-        <v>0.07006521776169702</v>
+        <v>0.07181581772532593</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -3664,10 +3664,10 @@
         </is>
       </c>
       <c r="B90">
-        <v>31.71726693386335</v>
+        <v>31.45441324706886</v>
       </c>
       <c r="C90">
-        <v>0.7926932346847683</v>
+        <v>0.796135816567096</v>
       </c>
       <c r="D90">
         <v>698.0405405405405</v>
@@ -3676,7 +3676,7 @@
         <v>2000</v>
       </c>
       <c r="F90">
-        <v>0.04543757144721494</v>
+        <v>0.04506101210498686</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -3701,10 +3701,10 @@
         </is>
       </c>
       <c r="B91">
-        <v>14.22634587148631</v>
+        <v>14.50533847413503</v>
       </c>
       <c r="C91">
-        <v>0.422086311745653</v>
+        <v>0.413973484942176</v>
       </c>
       <c r="D91">
         <v>161.3108108108108</v>
@@ -3713,7 +3713,7 @@
         <v>2000</v>
       </c>
       <c r="F91">
-        <v>0.0881921416176583</v>
+        <v>0.08992167605646244</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3738,10 +3738,10 @@
         </is>
       </c>
       <c r="B92">
-        <v>25.33654668577623</v>
+        <v>23.48295127982832</v>
       </c>
       <c r="C92">
-        <v>0.9176153753199253</v>
+        <v>0.9326336662080039</v>
       </c>
       <c r="D92">
         <v>1211.402777777778</v>
@@ -3750,7 +3750,7 @@
         <v>5000</v>
       </c>
       <c r="F92">
-        <v>0.02091504753873366</v>
+        <v>0.01938492441209845</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3775,10 +3775,10 @@
         </is>
       </c>
       <c r="B93">
-        <v>28.23476146346768</v>
+        <v>24.53976949122141</v>
       </c>
       <c r="C93">
-        <v>0.7577219862889435</v>
+        <v>0.8191879345004115</v>
       </c>
       <c r="D93">
         <v>644.4583333333334</v>
@@ -3787,7 +3787,7 @@
         <v>5000</v>
       </c>
       <c r="F93">
-        <v>0.04381161667571114</v>
+        <v>0.03807813200939509</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3812,10 +3812,10 @@
         </is>
       </c>
       <c r="B94">
-        <v>24.77346763605695</v>
+        <v>22.01097911875425</v>
       </c>
       <c r="C94">
-        <v>0.6900297236482329</v>
+        <v>0.7581674181688415</v>
       </c>
       <c r="D94">
         <v>629.8243243243244</v>
@@ -3824,7 +3824,7 @@
         <v>5000</v>
       </c>
       <c r="F94">
-        <v>0.03933393277980161</v>
+        <v>0.03494780729907127</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -3849,10 +3849,10 @@
         </is>
       </c>
       <c r="B95">
-        <v>16.17481186992759</v>
+        <v>14.70791124639109</v>
       </c>
       <c r="C95">
-        <v>0.4970761487724895</v>
+        <v>0.5806906793105139</v>
       </c>
       <c r="D95">
         <v>176.1081081081081</v>
@@ -3861,7 +3861,7 @@
         <v>5000</v>
       </c>
       <c r="F95">
-        <v>0.09184592375496026</v>
+        <v>0.08351637755010288</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3886,10 +3886,10 @@
         </is>
       </c>
       <c r="B96">
-        <v>25.45722993460461</v>
+        <v>21.70875557462728</v>
       </c>
       <c r="C96">
-        <v>0.4867517753690707</v>
+        <v>0.6280931344905551</v>
       </c>
       <c r="D96">
         <v>560.4324324324324</v>
@@ -3898,7 +3898,7 @@
         <v>5000</v>
       </c>
       <c r="F96">
-        <v>0.04542426251834349</v>
+        <v>0.03873572319932531</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -3923,10 +3923,10 @@
         </is>
       </c>
       <c r="B97">
-        <v>21.64515171530489</v>
+        <v>19.45628924388401</v>
       </c>
       <c r="C97">
-        <v>0.8792925454861296</v>
+        <v>0.9073837108355408</v>
       </c>
       <c r="D97">
         <v>1077.837837837838</v>
@@ -3935,7 +3935,7 @@
         <v>5000</v>
       </c>
       <c r="F97">
-        <v>0.02008201137076933</v>
+        <v>0.01805122121423542</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3960,10 +3960,10 @@
         </is>
       </c>
       <c r="B98">
-        <v>22.10631667226151</v>
+        <v>19.98860807437589</v>
       </c>
       <c r="C98">
-        <v>0.9270022199201349</v>
+        <v>0.9429509530338784</v>
       </c>
       <c r="D98">
         <v>1331.351351351351</v>
@@ -3972,7 +3972,7 @@
         <v>5000</v>
       </c>
       <c r="F98">
-        <v>0.01660441974977012</v>
+        <v>0.01501377382768794</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         </is>
       </c>
       <c r="B99">
-        <v>46.99588462470093</v>
+        <v>42.53061784250828</v>
       </c>
       <c r="C99">
-        <v>0.7320073950751652</v>
+        <v>0.7861728546877362</v>
       </c>
       <c r="D99">
         <v>1606.959459459459</v>
@@ -4009,7 +4009,7 @@
         <v>5000</v>
       </c>
       <c r="F99">
-        <v>0.0292452210589738</v>
+        <v>0.02646651574944804</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -4034,10 +4034,10 @@
         </is>
       </c>
       <c r="B100">
-        <v>50.05246299474504</v>
+        <v>48.78792303888461</v>
       </c>
       <c r="C100">
-        <v>0.7083739675026482</v>
+        <v>0.7264199051578263</v>
       </c>
       <c r="D100">
         <v>1936.189189189189</v>
@@ -4046,7 +4046,7 @@
         <v>5000</v>
       </c>
       <c r="F100">
-        <v>0.02585101873009906</v>
+        <v>0.02519791108807675</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -4071,10 +4071,10 @@
         </is>
       </c>
       <c r="B101">
-        <v>55.64448022468687</v>
+        <v>48.97986150834207</v>
       </c>
       <c r="C101">
-        <v>0.8988760835618601</v>
+        <v>0.9236367756858402</v>
       </c>
       <c r="D101">
         <v>1444.905405405405</v>
@@ -4083,7 +4083,7 @@
         <v>5000</v>
       </c>
       <c r="F101">
-        <v>0.03851081186112276</v>
+        <v>0.03389831702830367</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -4108,10 +4108,10 @@
         </is>
       </c>
       <c r="B102">
-        <v>15.86070103626347</v>
+        <v>14.51628715450107</v>
       </c>
       <c r="C102">
-        <v>0.4311793816272323</v>
+        <v>0.5095911682584944</v>
       </c>
       <c r="D102">
         <v>185.3108108108108</v>
@@ -4120,7 +4120,7 @@
         <v>5000</v>
       </c>
       <c r="F102">
-        <v>0.08558972337807166</v>
+        <v>0.07833480999293221</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -4145,10 +4145,10 @@
         </is>
       </c>
       <c r="B103">
-        <v>25.92966116804728</v>
+        <v>24.03206844218367</v>
       </c>
       <c r="C103">
-        <v>0.8094748524498845</v>
+        <v>0.8359723649541601</v>
       </c>
       <c r="D103">
         <v>763.9324324324324</v>
@@ -4157,7 +4157,7 @@
         <v>5000</v>
       </c>
       <c r="F103">
-        <v>0.03394234891361375</v>
+        <v>0.03145836911998004</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -4182,10 +4182,10 @@
         </is>
       </c>
       <c r="B104">
-        <v>16.03803038863013</v>
+        <v>14.8908792350412</v>
       </c>
       <c r="C104">
-        <v>0.7768274009368924</v>
+        <v>0.8079210668878968</v>
       </c>
       <c r="D104">
         <v>179.5405405405405</v>
@@ -4194,7 +4194,7 @@
         <v>5000</v>
       </c>
       <c r="F104">
-        <v>0.08932818370906438</v>
+        <v>0.08293881253899209</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -4219,10 +4219,10 @@
         </is>
       </c>
       <c r="B105">
-        <v>23.82317406449517</v>
+        <v>21.51566597134377</v>
       </c>
       <c r="C105">
-        <v>0.89510712685663</v>
+        <v>0.9155181560815383</v>
       </c>
       <c r="D105">
         <v>1240.108108108108</v>
@@ -4231,7 +4231,7 @@
         <v>5000</v>
       </c>
       <c r="F105">
-        <v>0.01921056229592715</v>
+        <v>0.01734983089834625</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -4256,10 +4256,10 @@
         </is>
       </c>
       <c r="B106">
-        <v>25.88107843388834</v>
+        <v>23.06464220090727</v>
       </c>
       <c r="C106">
-        <v>0.8929066780249169</v>
+        <v>0.9182894644387942</v>
       </c>
       <c r="D106">
         <v>1222.675675675676</v>
@@ -4268,7 +4268,7 @@
         <v>5000</v>
       </c>
       <c r="F106">
-        <v>0.02116757448338532</v>
+        <v>0.01886407218182473</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -4293,10 +4293,10 @@
         </is>
       </c>
       <c r="B107">
-        <v>26.55686598153348</v>
+        <v>23.41528956408289</v>
       </c>
       <c r="C107">
-        <v>0.8851374188627252</v>
+        <v>0.9180918565863473</v>
       </c>
       <c r="D107">
         <v>1347</v>
@@ -4305,7 +4305,7 @@
         <v>5000</v>
       </c>
       <c r="F107">
-        <v>0.01971556494545916</v>
+        <v>0.01738328846628277</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -4330,10 +4330,10 @@
         </is>
       </c>
       <c r="B108">
-        <v>22.76559986091647</v>
+        <v>19.68256804611726</v>
       </c>
       <c r="C108">
-        <v>0.9030524924432743</v>
+        <v>0.9295621547685526</v>
       </c>
       <c r="D108">
         <v>1091.013513513514</v>
@@ -4342,7 +4342,7 @@
         <v>5000</v>
       </c>
       <c r="F108">
-        <v>0.02086646918570408</v>
+        <v>0.01804062718043819</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -4367,10 +4367,10 @@
         </is>
       </c>
       <c r="B109">
-        <v>33.16623738266938</v>
+        <v>29.69861979644852</v>
       </c>
       <c r="C109">
-        <v>0.6538947099825407</v>
+        <v>0.7196033110911084</v>
       </c>
       <c r="D109">
         <v>351.1486486486486</v>
@@ -4379,7 +4379,7 @@
         <v>5000</v>
       </c>
       <c r="F109">
-        <v>0.09445070488041309</v>
+        <v>0.08457563459446568</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -4404,10 +4404,10 @@
         </is>
       </c>
       <c r="B110">
-        <v>27.50759254175625</v>
+        <v>25.75303452671607</v>
       </c>
       <c r="C110">
-        <v>0.6897844785377589</v>
+        <v>0.7266104991890638</v>
       </c>
       <c r="D110">
         <v>506.5405405405405</v>
@@ -4416,7 +4416,7 @@
         <v>5000</v>
       </c>
       <c r="F110">
-        <v>0.05430481933865015</v>
+        <v>0.05084101363186931</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -4441,10 +4441,10 @@
         </is>
       </c>
       <c r="B111">
-        <v>14.27915477651737</v>
+        <v>13.12273858684518</v>
       </c>
       <c r="C111">
-        <v>0.5065982122316304</v>
+        <v>0.5718360291588401</v>
       </c>
       <c r="D111">
         <v>147.2027027027027</v>
@@ -4453,7 +4453,7 @@
         <v>5000</v>
       </c>
       <c r="F111">
-        <v>0.09700334650346876</v>
+        <v>0.08914740249945319</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -4478,10 +4478,10 @@
         </is>
       </c>
       <c r="B112">
-        <v>21.63050129917735</v>
+        <v>19.7631167399577</v>
       </c>
       <c r="C112">
-        <v>0.9092811177612918</v>
+        <v>0.9255948167830127</v>
       </c>
       <c r="D112">
         <v>1100.662162162162</v>
@@ -4490,7 +4490,7 @@
         <v>5000</v>
       </c>
       <c r="F112">
-        <v>0.01965226210437358</v>
+        <v>0.01795566107327125</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -4515,10 +4515,10 @@
         </is>
       </c>
       <c r="B113">
-        <v>81.17688692904682</v>
+        <v>82.17481764028624</v>
       </c>
       <c r="C113">
-        <v>0.6098565279225344</v>
+        <v>0.6082294308599316</v>
       </c>
       <c r="D113">
         <v>2402.175675675676</v>
@@ -4527,7 +4527,7 @@
         <v>5000</v>
       </c>
       <c r="F113">
-        <v>0.03379306840504646</v>
+        <v>0.03420849626960459</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -4552,10 +4552,10 @@
         </is>
       </c>
       <c r="B114">
-        <v>41.08957623626293</v>
+        <v>35.63491498853003</v>
       </c>
       <c r="C114">
-        <v>0.9107088511784042</v>
+        <v>0.934147614731815</v>
       </c>
       <c r="D114">
         <v>1028.351351351351</v>
@@ -4564,7 +4564,7 @@
         <v>5000</v>
       </c>
       <c r="F114">
-        <v>0.03995674842286863</v>
+        <v>0.03465247061882339</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -4589,10 +4589,10 @@
         </is>
       </c>
       <c r="B115">
-        <v>22.73008912745383</v>
+        <v>20.96649374268461</v>
       </c>
       <c r="C115">
-        <v>0.9132476241379694</v>
+        <v>0.9285992778347506</v>
       </c>
       <c r="D115">
         <v>1186.959459459459</v>
@@ -4601,7 +4601,7 @@
         <v>5000</v>
       </c>
       <c r="F115">
-        <v>0.01914984454296788</v>
+        <v>0.01766403525882235</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -4626,10 +4626,10 @@
         </is>
       </c>
       <c r="B116">
-        <v>26.51301555365004</v>
+        <v>24.19802068284872</v>
       </c>
       <c r="C116">
-        <v>0.5947995654176776</v>
+        <v>0.6519924339343163</v>
       </c>
       <c r="D116">
         <v>450.027027027027</v>
@@ -4638,7 +4638,7 @@
         <v>5000</v>
       </c>
       <c r="F116">
-        <v>0.0589142739466129</v>
+        <v>0.05377014985678955</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -4663,10 +4663,10 @@
         </is>
       </c>
       <c r="B117">
-        <v>19.44717583091541</v>
+        <v>17.3872445041892</v>
       </c>
       <c r="C117">
-        <v>0.922385184701777</v>
+        <v>0.9383762455105361</v>
       </c>
       <c r="D117">
         <v>1172.797297297297</v>
@@ -4675,7 +4675,7 @@
         <v>5000</v>
       </c>
       <c r="F117">
-        <v>0.01658187299350986</v>
+        <v>0.01482544728254233</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -4700,10 +4700,10 @@
         </is>
       </c>
       <c r="B118">
-        <v>11.01770815803563</v>
+        <v>10.21886668722291</v>
       </c>
       <c r="C118">
-        <v>0.4710670768259717</v>
+        <v>0.5264953358402935</v>
       </c>
       <c r="D118">
         <v>111.3108108108108</v>
@@ -4712,7 +4712,7 @@
         <v>5000</v>
       </c>
       <c r="F118">
-        <v>0.09898147428610377</v>
+        <v>0.09180479966668634</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -4737,10 +4737,10 @@
         </is>
       </c>
       <c r="B119">
-        <v>18.5348115423684</v>
+        <v>17.44458988622317</v>
       </c>
       <c r="C119">
-        <v>0.4319796778646941</v>
+        <v>0.4923497259503128</v>
       </c>
       <c r="D119">
         <v>264.6216216216216</v>
@@ -4749,7 +4749,7 @@
         <v>5000</v>
       </c>
       <c r="F119">
-        <v>0.07004269503295175</v>
+        <v>0.0659227684394094</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -4774,10 +4774,10 @@
         </is>
       </c>
       <c r="B120">
-        <v>28.53053878593981</v>
+        <v>25.87028283110712</v>
       </c>
       <c r="C120">
-        <v>0.833027683848778</v>
+        <v>0.86436633027183</v>
       </c>
       <c r="D120">
         <v>698.0405405405405</v>
@@ -4786,7 +4786,7 @@
         <v>5000</v>
       </c>
       <c r="F120">
-        <v>0.04087232349549019</v>
+        <v>0.0370612898945296</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -4811,10 +4811,10 @@
         </is>
       </c>
       <c r="B121">
-        <v>14.42562310390701</v>
+        <v>13.24553357542341</v>
       </c>
       <c r="C121">
-        <v>0.4031278996630511</v>
+        <v>0.4752201168365479</v>
       </c>
       <c r="D121">
         <v>161.3108108108108</v>
@@ -4823,7 +4823,7 @@
         <v>5000</v>
       </c>
       <c r="F121">
-        <v>0.08942750353431504</v>
+        <v>0.08211187773991224</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -4848,10 +4848,10 @@
         </is>
       </c>
       <c r="B122">
-        <v>19.1635280321497</v>
+        <v>20.6080390124282</v>
       </c>
       <c r="C122">
-        <v>0.956704343557202</v>
+        <v>0.9514560113556498</v>
       </c>
       <c r="D122">
         <v>1211.402777777778</v>
@@ -4860,7 +4860,7 @@
         <v>10000</v>
       </c>
       <c r="F122">
-        <v>0.01581928684966669</v>
+        <v>0.01701171517059917</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -4885,10 +4885,10 @@
         </is>
       </c>
       <c r="B123">
-        <v>20.3162658112265</v>
+        <v>22.3758382952796</v>
       </c>
       <c r="C123">
-        <v>0.880485372963027</v>
+        <v>0.8509499441786676</v>
       </c>
       <c r="D123">
         <v>644.4583333333334</v>
@@ -4897,7 +4897,7 @@
         <v>10000</v>
       </c>
       <c r="F123">
-        <v>0.03152456064326863</v>
+        <v>0.03472038010517297</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -4922,10 +4922,10 @@
         </is>
       </c>
       <c r="B124">
-        <v>18.2194798787645</v>
+        <v>19.93655677924836</v>
       </c>
       <c r="C124">
-        <v>0.8356812699699802</v>
+        <v>0.8037997626605078</v>
       </c>
       <c r="D124">
         <v>629.8243243243244</v>
@@ -4934,7 +4934,7 @@
         <v>10000</v>
       </c>
       <c r="F124">
-        <v>0.02892787587762724</v>
+        <v>0.03165415499097515</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -4959,10 +4959,10 @@
         </is>
       </c>
       <c r="B125">
-        <v>13.06786517093156</v>
+        <v>13.93792031993645</v>
       </c>
       <c r="C125">
-        <v>0.6766977039673301</v>
+        <v>0.6261677993356689</v>
       </c>
       <c r="D125">
         <v>176.1081081081081</v>
@@ -4971,7 +4971,7 @@
         <v>10000</v>
       </c>
       <c r="F125">
-        <v>0.074203654285523</v>
+        <v>0.0791441147694366</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -4996,10 +4996,10 @@
         </is>
       </c>
       <c r="B126">
-        <v>18.15588475032876</v>
+        <v>19.73577554505489</v>
       </c>
       <c r="C126">
-        <v>0.7511791970463284</v>
+        <v>0.6941380682853431</v>
       </c>
       <c r="D126">
         <v>560.4324324324324</v>
@@ -5008,7 +5008,7 @@
         <v>10000</v>
       </c>
       <c r="F126">
-        <v>0.03239620639285128</v>
+        <v>0.03521526307711376</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -5033,10 +5033,10 @@
         </is>
       </c>
       <c r="B127">
-        <v>16.79258892473141</v>
+        <v>17.69313332939507</v>
       </c>
       <c r="C127">
-        <v>0.9329464397887609</v>
+        <v>0.9241061487464577</v>
       </c>
       <c r="D127">
         <v>1077.837837837838</v>
@@ -5045,7 +5045,7 @@
         <v>10000</v>
       </c>
       <c r="F127">
-        <v>0.01557988440860236</v>
+        <v>0.01641539451323012</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -5070,10 +5070,10 @@
         </is>
       </c>
       <c r="B128">
-        <v>17.85032022231935</v>
+        <v>19.04289682021802</v>
       </c>
       <c r="C128">
-        <v>0.9548117821741382</v>
+        <v>0.9472173449357132</v>
       </c>
       <c r="D128">
         <v>1331.351351351351</v>
@@ -5082,7 +5082,7 @@
         <v>10000</v>
       </c>
       <c r="F128">
-        <v>0.01340767048773479</v>
+        <v>0.01430343447722425</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -5107,10 +5107,10 @@
         </is>
       </c>
       <c r="B129">
-        <v>40.81398169900254</v>
+        <v>42.56427582707325</v>
       </c>
       <c r="C129">
-        <v>0.8029460994195263</v>
+        <v>0.7825952983593668</v>
       </c>
       <c r="D129">
         <v>1606.959459459459</v>
@@ -5119,7 +5119,7 @@
         <v>10000</v>
       </c>
       <c r="F129">
-        <v>0.02539826469096572</v>
+        <v>0.02648746088553522</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -5144,10 +5144,10 @@
         </is>
       </c>
       <c r="B130">
-        <v>47.36608836063551</v>
+        <v>47.77797168704121</v>
       </c>
       <c r="C130">
-        <v>0.7441407461406081</v>
+        <v>0.7392478539354018</v>
       </c>
       <c r="D130">
         <v>1936.189189189189</v>
@@ -5156,7 +5156,7 @@
         <v>10000</v>
       </c>
       <c r="F130">
-        <v>0.02446356411093837</v>
+        <v>0.02467629297478363</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -5181,10 +5181,10 @@
         </is>
       </c>
       <c r="B131">
-        <v>44.18104374915705</v>
+        <v>47.77430373358026</v>
       </c>
       <c r="C131">
-        <v>0.9386327969873283</v>
+        <v>0.9267504114333102</v>
       </c>
       <c r="D131">
         <v>1444.905405405405</v>
@@ -5193,7 +5193,7 @@
         <v>10000</v>
       </c>
       <c r="F131">
-        <v>0.03057711846317089</v>
+        <v>0.03306396637098603</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -5218,10 +5218,10 @@
         </is>
       </c>
       <c r="B132">
-        <v>13.42808052311803</v>
+        <v>14.29943609384425</v>
       </c>
       <c r="C132">
-        <v>0.5777817962537776</v>
+        <v>0.5245923551882982</v>
       </c>
       <c r="D132">
         <v>185.3108108108108</v>
@@ -5230,7 +5230,7 @@
         <v>10000</v>
       </c>
       <c r="F132">
-        <v>0.07246247784662251</v>
+        <v>0.07716460810504443</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -5255,10 +5255,10 @@
         </is>
       </c>
       <c r="B133">
-        <v>20.41907676902273</v>
+        <v>22.48720172934966</v>
       </c>
       <c r="C133">
-        <v>0.8828301913817632</v>
+        <v>0.8566134735789308</v>
       </c>
       <c r="D133">
         <v>763.9324324324324</v>
@@ -5267,7 +5267,7 @@
         <v>10000</v>
       </c>
       <c r="F133">
-        <v>0.0267289041571471</v>
+        <v>0.02943611342399523</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -5292,10 +5292,10 @@
         </is>
       </c>
       <c r="B134">
-        <v>12.85181956879516</v>
+        <v>14.10936972275139</v>
       </c>
       <c r="C134">
-        <v>0.8587380759808046</v>
+        <v>0.8281683558379829</v>
       </c>
       <c r="D134">
         <v>179.5405405405405</v>
@@ -5304,7 +5304,7 @@
         <v>10000</v>
       </c>
       <c r="F134">
-        <v>0.07158171369041408</v>
+        <v>0.07858598219807339</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -5329,10 +5329,10 @@
         </is>
       </c>
       <c r="B135">
-        <v>17.90345849842348</v>
+        <v>20.04237451665426</v>
       </c>
       <c r="C135">
-        <v>0.9426103838571761</v>
+        <v>0.9284802130570101</v>
       </c>
       <c r="D135">
         <v>1240.108108108108</v>
@@ -5341,7 +5341,7 @@
         <v>10000</v>
       </c>
       <c r="F135">
-        <v>0.01443701430654844</v>
+        <v>0.01616179620600226</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -5366,10 +5366,10 @@
         </is>
       </c>
       <c r="B136">
-        <v>19.34402729422667</v>
+        <v>21.50103432478701</v>
       </c>
       <c r="C136">
-        <v>0.9436910542969721</v>
+        <v>0.929857030213429</v>
       </c>
       <c r="D136">
         <v>1222.675675675676</v>
@@ -5378,7 +5378,7 @@
         <v>10000</v>
       </c>
       <c r="F136">
-        <v>0.01582106169204418</v>
+        <v>0.01758523110628262</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -5403,10 +5403,10 @@
         </is>
       </c>
       <c r="B137">
-        <v>19.97040197654702</v>
+        <v>21.98353026581539</v>
       </c>
       <c r="C137">
-        <v>0.9422293683106963</v>
+        <v>0.9275522559375604</v>
       </c>
       <c r="D137">
         <v>1347</v>
@@ -5415,7 +5415,7 @@
         <v>10000</v>
       </c>
       <c r="F137">
-        <v>0.0148258366566793</v>
+        <v>0.01632036396868254</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -5440,10 +5440,10 @@
         </is>
       </c>
       <c r="B138">
-        <v>16.50084445022647</v>
+        <v>18.72658922260702</v>
       </c>
       <c r="C138">
-        <v>0.9514523477133036</v>
+        <v>0.935286560250408</v>
       </c>
       <c r="D138">
         <v>1091.013513513514</v>
@@ -5452,7 +5452,7 @@
         <v>10000</v>
       </c>
       <c r="F138">
-        <v>0.01512432636795391</v>
+        <v>0.01716439713225886</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -5477,10 +5477,10 @@
         </is>
       </c>
       <c r="B139">
-        <v>26.01021409928804</v>
+        <v>28.49777808899296</v>
       </c>
       <c r="C139">
-        <v>0.785211728015626</v>
+        <v>0.7399034613426383</v>
       </c>
       <c r="D139">
         <v>351.1486486486486</v>
@@ -5489,7 +5489,7 @@
         <v>10000</v>
       </c>
       <c r="F139">
-        <v>0.07407180463141486</v>
+        <v>0.08115588141564284</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -5514,10 +5514,10 @@
         </is>
       </c>
       <c r="B140">
-        <v>21.71033032627709</v>
+        <v>23.87869021187534</v>
       </c>
       <c r="C140">
-        <v>0.8077447632512544</v>
+        <v>0.7646643197038533</v>
       </c>
       <c r="D140">
         <v>506.5405405405405</v>
@@ -5526,7 +5526,7 @@
         <v>10000</v>
       </c>
       <c r="F140">
-        <v>0.04286000544617716</v>
+        <v>0.04714072872902507</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -5551,10 +5551,10 @@
         </is>
       </c>
       <c r="B141">
-        <v>11.59452053331437</v>
+        <v>12.68251183271602</v>
       </c>
       <c r="C141">
-        <v>0.6758585560623191</v>
+        <v>0.6033846662783214</v>
       </c>
       <c r="D141">
         <v>147.2027027027027</v>
@@ -5563,7 +5563,7 @@
         <v>10000</v>
       </c>
       <c r="F141">
-        <v>0.07876567699121115</v>
+        <v>0.08615678652538193</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -5588,10 +5588,10 @@
         </is>
       </c>
       <c r="B142">
-        <v>16.74938190596345</v>
+        <v>17.83085441099693</v>
       </c>
       <c r="C142">
-        <v>0.9492735445788892</v>
+        <v>0.9408559324930762</v>
       </c>
       <c r="D142">
         <v>1100.662162162162</v>
@@ -5600,7 +5600,7 @@
         <v>10000</v>
       </c>
       <c r="F142">
-        <v>0.01521755038172716</v>
+        <v>0.01620011573394115</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -5625,10 +5625,10 @@
         </is>
       </c>
       <c r="B143">
-        <v>84.31686436791549</v>
+        <v>80.73235436703081</v>
       </c>
       <c r="C143">
-        <v>0.5810322352873744</v>
+        <v>0.6113486914799645</v>
       </c>
       <c r="D143">
         <v>2402.175675675676</v>
@@ -5637,7 +5637,7 @@
         <v>10000</v>
       </c>
       <c r="F143">
-        <v>0.03510020737521585</v>
+        <v>0.03360801426162251</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -5662,10 +5662,10 @@
         </is>
       </c>
       <c r="B144">
-        <v>28.92048621382486</v>
+        <v>31.73368188746328</v>
       </c>
       <c r="C144">
-        <v>0.9581089829485609</v>
+        <v>0.9486275651005184</v>
       </c>
       <c r="D144">
         <v>1028.351351351351</v>
@@ -5674,7 +5674,7 @@
         <v>10000</v>
       </c>
       <c r="F144">
-        <v>0.02812315671664222</v>
+        <v>0.0308587933936803</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -5699,10 +5699,10 @@
         </is>
       </c>
       <c r="B145">
-        <v>17.41169235899434</v>
+        <v>18.76076842828314</v>
       </c>
       <c r="C145">
-        <v>0.955080744106012</v>
+        <v>0.9456302332269145</v>
       </c>
       <c r="D145">
         <v>1186.959459459459</v>
@@ -5711,7 +5711,7 @@
         <v>10000</v>
       </c>
       <c r="F145">
-        <v>0.01466915505852543</v>
+        <v>0.01580573647968296</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -5736,10 +5736,10 @@
         </is>
       </c>
       <c r="B146">
-        <v>21.83425129487189</v>
+        <v>23.32088505493221</v>
       </c>
       <c r="C146">
-        <v>0.7120695039096611</v>
+        <v>0.6741081335945378</v>
       </c>
       <c r="D146">
         <v>450.027027027027</v>
@@ -5748,7 +5748,7 @@
         <v>10000</v>
       </c>
       <c r="F146">
-        <v>0.04851764446040837</v>
+        <v>0.05182107663398545</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -5773,10 +5773,10 @@
         </is>
       </c>
       <c r="B147">
-        <v>15.23890065245767</v>
+        <v>16.14656590689415</v>
       </c>
       <c r="C147">
-        <v>0.9533366727551134</v>
+        <v>0.9477214215086833</v>
       </c>
       <c r="D147">
         <v>1172.797297297297</v>
@@ -5785,7 +5785,7 @@
         <v>10000</v>
       </c>
       <c r="F147">
-        <v>0.0129936355477418</v>
+        <v>0.01376756745952927</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -5810,10 +5810,10 @@
         </is>
       </c>
       <c r="B148">
-        <v>9.020486745612871</v>
+        <v>9.915593484017061</v>
       </c>
       <c r="C148">
-        <v>0.6283313950144245</v>
+        <v>0.5502982375288072</v>
       </c>
       <c r="D148">
         <v>111.3108108108108</v>
@@ -5822,7 +5822,7 @@
         <v>10000</v>
       </c>
       <c r="F148">
-        <v>0.08103873002007436</v>
+        <v>0.08908023768571841</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -5847,10 +5847,10 @@
         </is>
       </c>
       <c r="B149">
-        <v>16.05422526831881</v>
+        <v>17.33862773010066</v>
       </c>
       <c r="C149">
-        <v>0.5698888245023813</v>
+        <v>0.4951523860447896</v>
       </c>
       <c r="D149">
         <v>264.6216216216216</v>
@@ -5859,7 +5859,7 @@
         <v>10000</v>
       </c>
       <c r="F149">
-        <v>0.0606686073871715</v>
+        <v>0.06552233949685675</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -5884,10 +5884,10 @@
         </is>
       </c>
       <c r="B150">
-        <v>21.69222000015406</v>
+        <v>23.92599936317805</v>
       </c>
       <c r="C150">
-        <v>0.9072082345923796</v>
+        <v>0.8857918338886452</v>
       </c>
       <c r="D150">
         <v>698.0405405405405</v>
@@ -5896,7 +5896,7 @@
         <v>10000</v>
       </c>
       <c r="F150">
-        <v>0.03107587416535476</v>
+        <v>0.03427594526909642</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -5921,10 +5921,10 @@
         </is>
       </c>
       <c r="B151">
-        <v>11.32333460160206</v>
+        <v>12.58232325562051</v>
       </c>
       <c r="C151">
-        <v>0.6198659056498341</v>
+        <v>0.525222216250274</v>
       </c>
       <c r="D151">
         <v>161.3108108108108</v>
@@ -5933,7 +5933,7 @@
         <v>10000</v>
       </c>
       <c r="F151">
-        <v>0.07019575777151314</v>
+        <v>0.07800049601373191</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>

</xml_diff>